<commit_message>
working for validation Branch Division Fin Year with data provider
</commit_message>
<xml_diff>
--- a/src/test/resources/TestByDataprovider.xlsx
+++ b/src/test/resources/TestByDataprovider.xlsx
@@ -4,18 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
-    <sheet name="BranchSheet" sheetId="2" r:id="rId2"/>
+    <sheet name="BranchSheetWith_ID" sheetId="2" r:id="rId2"/>
+    <sheet name="All_BranchSheet" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="28">
   <si>
     <t>username</t>
   </si>
@@ -440,7 +441,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -634,4 +635,118 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updating : Read method in excel and validate login through title with valid and invalid credentials
</commit_message>
<xml_diff>
--- a/src/test/resources/TestByDataprovider.xlsx
+++ b/src/test/resources/TestByDataprovider.xlsx
@@ -4,19 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
-    <sheet name="BranchSheetWith_ID" sheetId="2" r:id="rId2"/>
-    <sheet name="All_BranchSheet" sheetId="3" r:id="rId3"/>
+    <sheet name="All_BranchSheet" sheetId="3" r:id="rId2"/>
+    <sheet name="BranchSheetWith_ID" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="34">
   <si>
     <t>username</t>
   </si>
@@ -100,6 +100,24 @@
   </si>
   <si>
     <t>ID-8</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>expectedTitle</t>
+  </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t>Valid</t>
+  </si>
+  <si>
+    <t>iCaffe</t>
+  </si>
+  <si>
+    <t>Login Branch Division</t>
   </si>
 </sst>
 </file>
@@ -449,42 +467,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1">
         <v>123</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -497,6 +540,120 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -635,118 +792,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Flow of Login and Branch_Division_FinancialYear and Validation with Multiple Data taking by Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/TestByDataprovider.xlsx
+++ b/src/test/resources/TestByDataprovider.xlsx
@@ -4,19 +4,20 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
     <sheet name="All_BranchSheet" sheetId="3" r:id="rId2"/>
     <sheet name="BranchSheetWith_ID" sheetId="2" r:id="rId3"/>
+    <sheet name="MastersParty" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="49">
   <si>
     <t>username</t>
   </si>
@@ -51,9 +52,6 @@
     <t>optExportAir</t>
   </si>
   <si>
-    <t>2025-26</t>
-  </si>
-  <si>
     <t>Mumbai</t>
   </si>
   <si>
@@ -69,9 +67,6 @@
     <t>optImportSea</t>
   </si>
   <si>
-    <t>2024-25</t>
-  </si>
-  <si>
     <t>finYear</t>
   </si>
   <si>
@@ -118,13 +113,64 @@
   </si>
   <si>
     <t>Login Branch Division</t>
+  </si>
+  <si>
+    <t>Akash12</t>
+  </si>
+  <si>
+    <t>DEMO LTD</t>
+  </si>
+  <si>
+    <t>Mumbai (Export Air)</t>
+  </si>
+  <si>
+    <t>exp_4</t>
+  </si>
+  <si>
+    <t>Mumbai (Export Sea)</t>
+  </si>
+  <si>
+    <t>Mumbai (Import Air)</t>
+  </si>
+  <si>
+    <t>Mumbai (Import Sea)</t>
+  </si>
+  <si>
+    <t>(2627)</t>
+  </si>
+  <si>
+    <t>Ahmedabad (Export Air)</t>
+  </si>
+  <si>
+    <t>Ahmedabad (Export Sea)</t>
+  </si>
+  <si>
+    <t>Ahmedabad (Import Air)</t>
+  </si>
+  <si>
+    <t>Ahmedabad (Import Sea)</t>
+  </si>
+  <si>
+    <t>exp_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exp_2 </t>
+  </si>
+  <si>
+    <t>exp_3</t>
+  </si>
+  <si>
+    <t>Shipper Master</t>
+  </si>
+  <si>
+    <t>valid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -152,6 +198,11 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -174,7 +225,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -186,6 +237,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -459,7 +511,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -482,10 +534,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -496,10 +548,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
         <v>30</v>
-      </c>
-      <c r="D2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -510,10 +562,10 @@
         <v>123</v>
       </c>
       <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
         <v>30</v>
-      </c>
-      <c r="D3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -524,10 +576,10 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
         <v>31</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -541,15 +593,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -557,54 +613,114 @@
         <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
       <c r="C5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -612,40 +728,88 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -661,11 +825,15 @@
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>7</v>
@@ -674,68 +842,68 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -744,49 +912,78 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Validation For Login Test Case and Update some of method for Naming convention for Report Reading purpose. Validate Branch, Division and Financial Year Selection For all Cases. Update Autosuggest Method in Webutil class for Autosuggesting Textbox.
</commit_message>
<xml_diff>
--- a/src/test/resources/TestByDataprovider.xlsx
+++ b/src/test/resources/TestByDataprovider.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
-    <sheet name="BranchSheet" sheetId="2" r:id="rId2"/>
-    <sheet name="CFSMasterSheet" sheetId="3" r:id="rId3"/>
+    <sheet name="All_BranchSheet" sheetId="2" r:id="rId2"/>
+    <sheet name="BranchSheetWith_ID" sheetId="4" r:id="rId3"/>
+    <sheet name="BankBROSheet" sheetId="5" r:id="rId4"/>
+    <sheet name="CFSMasterSheet" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="59">
   <si>
     <t>username</t>
   </si>
@@ -57,17 +59,149 @@
     <t>ZAZDV</t>
   </si>
   <si>
-    <t>ABC BY Excel Automation</t>
-  </si>
-  <si>
-    <t>xyz By shivam</t>
+    <t>type</t>
+  </si>
+  <si>
+    <t>expectedTitle</t>
+  </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t>iCaffe</t>
+  </si>
+  <si>
+    <t>Valid</t>
+  </si>
+  <si>
+    <t>Login Branch Division</t>
+  </si>
+  <si>
+    <t>shivam</t>
+  </si>
+  <si>
+    <t>singh</t>
+  </si>
+  <si>
+    <t>icaffe</t>
+  </si>
+  <si>
+    <t>hans</t>
+  </si>
+  <si>
+    <t>xyz</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>optExportAir</t>
+  </si>
+  <si>
+    <t>optImportAir</t>
+  </si>
+  <si>
+    <t>optImportSea</t>
+  </si>
+  <si>
+    <t>ID-1</t>
+  </si>
+  <si>
+    <t>2025-26</t>
+  </si>
+  <si>
+    <t>ID-2</t>
+  </si>
+  <si>
+    <t>ID-3</t>
+  </si>
+  <si>
+    <t>2024-25</t>
+  </si>
+  <si>
+    <t>ID-4</t>
+  </si>
+  <si>
+    <t>ID-5</t>
+  </si>
+  <si>
+    <t>ID-6</t>
+  </si>
+  <si>
+    <t>ID-7</t>
+  </si>
+  <si>
+    <t>ID-8</t>
+  </si>
+  <si>
+    <t>expDataID</t>
+  </si>
+  <si>
+    <t>infomatic</t>
+  </si>
+  <si>
+    <t>at</t>
+  </si>
+  <si>
+    <t>amit@123</t>
+  </si>
+  <si>
+    <t>bankName</t>
+  </si>
+  <si>
+    <t>branchName</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>Kerala</t>
+  </si>
+  <si>
+    <t>Rajasthan</t>
+  </si>
+  <si>
+    <t>Automation Testing 30 1</t>
+  </si>
+  <si>
+    <t>Automation Testing 30 2</t>
+  </si>
+  <si>
+    <t>CZLOB</t>
+  </si>
+  <si>
+    <t>Automation Testing 30 3</t>
+  </si>
+  <si>
+    <t>FRC3S</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Excel bank 8</t>
+  </si>
+  <si>
+    <t>excel branch 8</t>
+  </si>
+  <si>
+    <t>Excel bank 9</t>
+  </si>
+  <si>
+    <t>excel branch 9</t>
+  </si>
+  <si>
+    <t>Excel bank 10</t>
+  </si>
+  <si>
+    <t>excel branch 10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -102,6 +236,14 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -124,17 +266,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -142,14 +303,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -416,31 +569,130 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
+      <c r="C1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="5" customFormat="1">
+      <c r="A4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>123</v>
+      </c>
+      <c r="B8">
+        <v>123</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B5" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId2"/>
@@ -449,32 +701,110 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
+      <c r="A1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="A2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C7" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>6</v>
       </c>
     </row>
@@ -485,35 +815,274 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="38.140625" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.75">
+      <c r="A1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="8" customFormat="1">
+      <c r="C5"/>
+    </row>
+    <row r="6" spans="1:3" s="8" customFormat="1"/>
+    <row r="7" spans="1:3" s="8" customFormat="1"/>
+    <row r="8" spans="1:3" s="8" customFormat="1"/>
+    <row r="9" spans="1:3" s="8" customFormat="1"/>
+    <row r="10" spans="1:3" s="8" customFormat="1"/>
+    <row r="12" spans="1:3">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="13"/>
+      <c r="B15" s="12"/>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="13"/>
+      <c r="B16" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="29.85546875" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" ht="15.75">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="5" t="s">
+      <c r="C1" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75">
+      <c r="A2" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>12</v>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75">
+      <c r="A3" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75">
+      <c r="A4" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CFS Master Page working
</commit_message>
<xml_diff>
--- a/src/test/resources/TestByDataprovider.xlsx
+++ b/src/test/resources/TestByDataprovider.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="92">
   <si>
     <t>username</t>
   </si>
@@ -155,24 +155,9 @@
     <t>state</t>
   </si>
   <si>
-    <t>Kerala</t>
-  </si>
-  <si>
-    <t>Rajasthan</t>
-  </si>
-  <si>
-    <t>Automation Testing 30 1</t>
-  </si>
-  <si>
-    <t>Automation Testing 30 2</t>
-  </si>
-  <si>
     <t>CZLOB</t>
   </si>
   <si>
-    <t>Automation Testing 30 3</t>
-  </si>
-  <si>
     <t>FRC3S</t>
   </si>
   <si>
@@ -195,6 +180,120 @@
   </si>
   <si>
     <t>excel branch 10</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>address1</t>
+  </si>
+  <si>
+    <t>address2</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>zipcode</t>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>fax</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>pan</t>
+  </si>
+  <si>
+    <t>ediGroupCode</t>
+  </si>
+  <si>
+    <t>bondValue</t>
+  </si>
+  <si>
+    <t>Sending Data By Excel 1</t>
+  </si>
+  <si>
+    <t>Sending Data By Excel 2</t>
+  </si>
+  <si>
+    <t>Sending Data By Excel 3</t>
+  </si>
+  <si>
+    <t>A-01</t>
+  </si>
+  <si>
+    <t>A-02</t>
+  </si>
+  <si>
+    <t>A-03</t>
+  </si>
+  <si>
+    <t>Noida</t>
+  </si>
+  <si>
+    <t>Sector-01</t>
+  </si>
+  <si>
+    <t>Sector-02</t>
+  </si>
+  <si>
+    <t>Sector-03</t>
+  </si>
+  <si>
+    <t>Uttar Pradesh</t>
+  </si>
+  <si>
+    <t>123-456789</t>
+  </si>
+  <si>
+    <t>456-789012</t>
+  </si>
+  <si>
+    <t>789-123456</t>
+  </si>
+  <si>
+    <t>test1@gmail.com</t>
+  </si>
+  <si>
+    <t>test2@gmail.com</t>
+  </si>
+  <si>
+    <t>test3@gmail.com</t>
+  </si>
+  <si>
+    <t>ABCDE1234L</t>
+  </si>
+  <si>
+    <t>XYZAS1234F</t>
+  </si>
+  <si>
+    <t>FGHIJ1234T</t>
+  </si>
+  <si>
+    <t>EGV01</t>
+  </si>
+  <si>
+    <t>EGV02</t>
+  </si>
+  <si>
+    <t>EGV03</t>
+  </si>
+  <si>
+    <t>BV01</t>
+  </si>
+  <si>
+    <t>BV02</t>
+  </si>
+  <si>
+    <t>BV03</t>
   </si>
 </sst>
 </file>
@@ -237,12 +336,11 @@
       <family val="3"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -266,7 +364,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -289,13 +387,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -561,7 +654,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -957,7 +1050,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -965,7 +1058,7 @@
     <col min="3" max="3" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75">
+    <row r="1" spans="1:2" ht="15.75">
       <c r="A1" s="3" t="s">
         <v>42</v>
       </c>
@@ -973,57 +1066,29 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:2">
       <c r="A2" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="8" customFormat="1">
-      <c r="C5"/>
-    </row>
-    <row r="6" spans="1:3" s="8" customFormat="1"/>
-    <row r="7" spans="1:3" s="8" customFormat="1"/>
-    <row r="8" spans="1:3" s="8" customFormat="1"/>
-    <row r="9" spans="1:3" s="8" customFormat="1"/>
-    <row r="10" spans="1:3" s="8" customFormat="1"/>
-    <row r="12" spans="1:3">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="12"/>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1033,60 +1098,220 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="29.85546875" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
     <col min="3" max="3" width="21.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="8" max="8" width="18.140625" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="11" width="19.140625" customWidth="1"/>
+    <col min="12" max="12" width="25" customWidth="1"/>
+    <col min="13" max="13" width="21.85546875" customWidth="1"/>
+    <col min="14" max="14" width="20.85546875" customWidth="1"/>
+    <col min="15" max="15" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75">
+    <row r="1" spans="1:15" ht="15.75">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75">
+      <c r="H1" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="O1" s="12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="15.75">
       <c r="A2" s="8" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2">
+        <v>201301</v>
+      </c>
+      <c r="I2">
+        <v>1234567890</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="K2">
+        <v>123456</v>
+      </c>
+      <c r="L2" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="15.75">
+      <c r="A3" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75">
-      <c r="A3" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="C3" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3">
+        <v>200300</v>
+      </c>
+      <c r="I3">
+        <v>9876543210</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="K3">
+        <v>7890123</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="15.75">
+      <c r="A4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.75">
-      <c r="A4" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="C4" s="8" t="s">
-        <v>52</v>
+        <v>71</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H4">
+        <v>201301</v>
+      </c>
+      <c r="I4" s="8">
+        <v>1234567890</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="K4">
+        <v>3698520</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="L2" r:id="rId1"/>
+    <hyperlink ref="L3" r:id="rId2"/>
+    <hyperlink ref="L4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>